<commit_message>
Build site at 2021-04-23 14:32:26 UTC
</commit_message>
<xml_diff>
--- a/_Drive/Publicacoes/Publicacoes.xlsx
+++ b/_Drive/Publicacoes/Publicacoes.xlsx
@@ -9,46 +9,82 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion1">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataSignature="AMtx7mgvS8o56TleT807myZNmcBSuuuW5g=="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataSignature="AMtx7mg0x8YA1UjSz3556HCLQEhKJFMWiA=="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>DOI</t>
   </si>
   <si>
+    <t>10.1007/s11669-019-00756-6</t>
+  </si>
+  <si>
+    <t>10.1007/s42452-019-1479-z</t>
+  </si>
+  <si>
+    <t>10.1016/j.calphad.2018.05.004</t>
+  </si>
+  <si>
+    <t>10.1016/j.calphad.2019.101676</t>
+  </si>
+  <si>
+    <t>10.1016/j.calphad.2019.101687</t>
+  </si>
+  <si>
+    <t>10.1016/j.ceramint.2020.11.013</t>
+  </si>
+  <si>
+    <t>10.1016/j.jallcom.2019.02.072</t>
+  </si>
+  <si>
+    <t>10.1016/j.jallcom.2019.06.186</t>
+  </si>
+  <si>
+    <t>10.1016/j.matchemphys.2017.03.037</t>
+  </si>
+  <si>
+    <t>10.1016/j.matchemphys.2019.01.008</t>
+  </si>
+  <si>
+    <t>10.1016/j.mtla.2018.11.008</t>
+  </si>
+  <si>
+    <t>10.1016/j.physleta.2018.02.018</t>
+  </si>
+  <si>
+    <t>10.1016/j.scriptamat.2021.113854</t>
+  </si>
+  <si>
+    <t>10.1016/j.ssc.2018.08.014</t>
+  </si>
+  <si>
     <t>10.1103/PhysRevB.103.125134</t>
   </si>
   <si>
-    <t>10.1016/j.scriptamat.2021.113854</t>
+    <t>10.1103/PhysRevB.95.094505</t>
+  </si>
+  <si>
+    <t>10.1103/PhysRevB.95.144505</t>
+  </si>
+  <si>
+    <t>10.1103/PhysRevB.96.014507</t>
+  </si>
+  <si>
+    <t>10.1103/physrevb.98.045126</t>
+  </si>
+  <si>
+    <t>10.1103/PhysRevLett.122.147001</t>
+  </si>
+  <si>
+    <t>10.1103/physrevmaterials.1.044803</t>
   </si>
   <si>
     <t>10.1103/PhysRevResearch.2.022001</t>
-  </si>
-  <si>
-    <t>10.1016/j.calphad.2019.101676</t>
-  </si>
-  <si>
-    <t>10.1016/j.calphad.2019.101687</t>
-  </si>
-  <si>
-    <t>10.1016/j.ssc.2018.08.014</t>
-  </si>
-  <si>
-    <t>10.1016/j.mtla.2018.11.008</t>
-  </si>
-  <si>
-    <t>10.1103/physrevb.98.045126</t>
-  </si>
-  <si>
-    <t>10.1016/j.calphad.2018.05.004</t>
-  </si>
-  <si>
-    <t>10.1103/PhysRevB.95.144505</t>
   </si>
 </sst>
 </file>
@@ -66,9 +102,12 @@
       <color rgb="FF000000"/>
     </font>
     <font>
-      <color rgb="FF000000"/>
+      <name val="Helvetica"/>
     </font>
-    <font/>
+    <font>
+      <color theme="1"/>
+      <name val="Helvetica"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -84,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -92,11 +131,12 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+      <alignment horizontal="left" readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+      <alignment horizontal="left" readingOrder="0" vertical="bottom"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -323,64 +363,178 @@
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="4"/>
     </row>
     <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="4"/>
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="4"/>
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="4"/>
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="4"/>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="4"/>
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="4"/>
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="4"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
     </row>
     <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="12" ht="15.75" customHeight="1"/>
-    <row r="13" ht="15.75" customHeight="1"/>
-    <row r="14" ht="15.75" customHeight="1"/>
-    <row r="15" ht="15.75" customHeight="1"/>
-    <row r="16" ht="15.75" customHeight="1"/>
-    <row r="17" ht="15.75" customHeight="1"/>
-    <row r="18" ht="15.75" customHeight="1"/>
-    <row r="19" ht="15.75" customHeight="1"/>
-    <row r="20" ht="15.75" customHeight="1"/>
-    <row r="21" ht="15.75" customHeight="1"/>
-    <row r="22" ht="15.75" customHeight="1"/>
-    <row r="23" ht="15.75" customHeight="1"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+    </row>
+    <row r="12" ht="15.75" customHeight="1">
+      <c r="A12" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="4"/>
+    </row>
+    <row r="13" ht="15.75" customHeight="1">
+      <c r="A13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="4"/>
+    </row>
+    <row r="14" ht="15.75" customHeight="1">
+      <c r="A14" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+    </row>
+    <row r="15" ht="15.75" customHeight="1">
+      <c r="A15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="4"/>
+    </row>
+    <row r="16" ht="15.75" customHeight="1">
+      <c r="A16" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="4"/>
+    </row>
+    <row r="17" ht="15.75" customHeight="1">
+      <c r="A17" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="4"/>
+    </row>
+    <row r="18" ht="15.75" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="4"/>
+    </row>
+    <row r="19" ht="15.75" customHeight="1">
+      <c r="A19" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="4"/>
+    </row>
+    <row r="20" ht="15.75" customHeight="1">
+      <c r="A20" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="4"/>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+    </row>
     <row r="24" ht="15.75" customHeight="1"/>
     <row r="25" ht="15.75" customHeight="1"/>
     <row r="26" ht="15.75" customHeight="1"/>
@@ -1357,8 +1511,6 @@
     <row r="997" ht="15.75" customHeight="1"/>
     <row r="998" ht="15.75" customHeight="1"/>
     <row r="999" ht="15.75" customHeight="1"/>
-    <row r="1000" ht="15.75" customHeight="1"/>
-    <row r="1001" ht="15.75" customHeight="1"/>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>